<commit_message>
onboarding: match the app's "shared with bot" wording
The pull brought in 62815b6, which deliberately replaced "publish" /
"საჯარო" everywhere: for a bank or a clinic, "გამოაქვეყნეთ" read as
"made public on the internet" -- terrifying wording for a switch that
only controls what an internal bot may quote.

The intake form, written before that landed, reintroduced exactly the
word that was removed. A customer would have learned "საჯარო" from the
form and then never seen it again in the product.

Now uses the app's own strings verbatim -- "ბოტისთვის დაშვებული" /
"შიდა" -- in the dropdown, the examples and the explanation, and carries
the same reassurance the app gives ("ინტერნეტში არაფერი ქვეყნდება").
Widened the column, since the new label is far longer than the old one.

Verified against brand.js at build time and re-run through the real
csv_to_chunks: still one row per chunk.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/onboarding/dist/CommuniQ-AI-კითხვარი.xlsx
+++ b/onboarding/dist/CommuniQ-AI-კითხვარი.xlsx
@@ -1153,9 +1153,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="74" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1182,7 +1182,7 @@
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>ხილვადობა: „საჯარო“ — პასუხი შეიძლება სიტყვასიტყვით ეთქვას კლიენტს. „შიდა“ — მხოლოდ თანამშრომლებისთვის (შიდა წესები, ფასდაკლების ლიმიტები, ესკალაციის პირობები). თუ ეჭვობთ — აირჩიეთ „შიდა“.</t>
+          <t>ხილვადობა: „ბოტისთვის დაშვებული“ — ბოტს შეუძლია ეს პასუხი კლიენტს სიტყვასიტყვით მოახსენოს. „შიდა“ — მხოლოდ თანამშრომლებისთვის (შიდა წესები, ფასდაკლების ლიმიტები, ესკალაციის პირობები). თუ ეჭვობთ — აირჩიეთ „შიდა“. ინტერნეტში არაფერი ქვეყნდება — მონაცემები თქვენს სამუშაო სივრცეში რჩება.</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>საჯარო</t>
+          <t>ბოტისთვის დაშვებული</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>საჯარო</t>
+          <t>ბოტისთვის დაშვებული</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>საჯარო</t>
+          <t>ბოტისთვის დაშვებული</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>საჯარო</t>
+          <t>ბოტისთვის დაშვებული</t>
         </is>
       </c>
     </row>
@@ -1655,8 +1655,8 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="არასწორი მნიშვნელობა" error="აირჩიეთ „საჯარო“ ან „შიდა“." type="list">
-      <formula1>"საჯარო,შიდა"</formula1>
+    <dataValidation sqref="D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="არასწორი მნიშვნელობა" error="აირჩიეთ „ბოტისთვის დაშვებული“ ან „შიდა“." type="list">
+      <formula1>"ბოტისთვის დაშვებული,შიდა"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>